<commit_message>
resultados.py: profit factor e esperanca matematica (mesmo padrao do omqs_api)
_resumo() agora usa _metricas(), compartilhada: alem de acerto/retorno,
calcula profit_factor (soma ganhos/|soma perdas|) e esperanca_matematica
(acerto*ganho_medio - (1-acerto)*|perda_media|).

Achado (11/08, N=11): profit factor geral 0.03 -- pior ainda que o
retorno medio ja sugeria. Compra (N=5): PF 0.00, nenhum trade positivo.
Venda (N=6): PF 0.15, um pouco menos ruim.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/resultados/resultados_2026_08_11.xlsx
+++ b/resultados/resultados_2026_08_11.xlsx
@@ -1262,7 +1262,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:E4"/>
+  <dimension ref="A1:I4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1291,6 +1291,26 @@
           <t>retorno_total</t>
         </is>
       </c>
+      <c r="F1" t="inlineStr">
+        <is>
+          <t>ganho_medio</t>
+        </is>
+      </c>
+      <c r="G1" t="inlineStr">
+        <is>
+          <t>perda_media</t>
+        </is>
+      </c>
+      <c r="H1" t="inlineStr">
+        <is>
+          <t>profit_factor</t>
+        </is>
+      </c>
+      <c r="I1" t="inlineStr">
+        <is>
+          <t>esperanca_matematica</t>
+        </is>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1310,6 +1330,18 @@
       <c r="E2" t="n">
         <v>-0.2584</v>
       </c>
+      <c r="F2" t="n">
+        <v>0.0046</v>
+      </c>
+      <c r="G2" t="n">
+        <v>-0.0297</v>
+      </c>
+      <c r="H2" t="n">
+        <v>0.034</v>
+      </c>
+      <c r="I2" t="n">
+        <v>-0.0235</v>
+      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1329,6 +1361,18 @@
       <c r="E3" t="n">
         <v>-0.208</v>
       </c>
+      <c r="F3" t="n">
+        <v>0</v>
+      </c>
+      <c r="G3" t="n">
+        <v>-0.0416</v>
+      </c>
+      <c r="H3" t="n">
+        <v>0</v>
+      </c>
+      <c r="I3" t="n">
+        <v>-0.0416</v>
+      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1347,6 +1391,18 @@
       </c>
       <c r="E4" t="n">
         <v>-0.0504</v>
+      </c>
+      <c r="F4" t="n">
+        <v>0.0046</v>
+      </c>
+      <c r="G4" t="n">
+        <v>-0.0149</v>
+      </c>
+      <c r="H4" t="n">
+        <v>0.153</v>
+      </c>
+      <c r="I4" t="n">
+        <v>-0.008399999999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
resultados.py: remove esperanca_matematica (redundante com retorno_medio)
Mesmo motivo do omqs_api: com trades de tamanho uniforme, esperanca
matematica e identica a retorno_medio. Mantidos ganho_medio, perda_media
e profit_factor.

Co-Authored-By: Claude Sonnet 5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/resultados/resultados_2026_08_11.xlsx
+++ b/resultados/resultados_2026_08_11.xlsx
@@ -1262,7 +1262,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I4"/>
+  <dimension ref="A1:H4"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <sheetData>
     <row r="1">
@@ -1306,11 +1306,6 @@
           <t>profit_factor</t>
         </is>
       </c>
-      <c r="I1" t="inlineStr">
-        <is>
-          <t>esperanca_matematica</t>
-        </is>
-      </c>
     </row>
     <row r="2">
       <c r="A2" t="inlineStr">
@@ -1339,9 +1334,6 @@
       <c r="H2" t="n">
         <v>0.034</v>
       </c>
-      <c r="I2" t="n">
-        <v>-0.0235</v>
-      </c>
     </row>
     <row r="3">
       <c r="A3" t="inlineStr">
@@ -1370,9 +1362,6 @@
       <c r="H3" t="n">
         <v>0</v>
       </c>
-      <c r="I3" t="n">
-        <v>-0.0416</v>
-      </c>
     </row>
     <row r="4">
       <c r="A4" t="inlineStr">
@@ -1400,9 +1389,6 @@
       </c>
       <c r="H4" t="n">
         <v>0.153</v>
-      </c>
-      <c r="I4" t="n">
-        <v>-0.008399999999999999</v>
       </c>
     </row>
   </sheetData>

</xml_diff>